<commit_message>
fixed bug in reg_education.xlsx
</commit_message>
<xml_diff>
--- a/input/reg_education.xlsx
+++ b/input/reg_education.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Patryk\git\SimPaths_HU\input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/pineapple/IdeaProjects/ESPONmodels/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06213481-F875-47C4-A649-318919CF0EDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CDE477F8-1D5B-0C4C-9B03-68300D726D84}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="28996" windowHeight="17475" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="30240" windowHeight="18880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="42">
   <si>
     <t>Description:</t>
   </si>
@@ -145,14 +145,17 @@
     <t>Year_transformed_</t>
   </si>
   <si>
-    <t>Dag_</t>
+    <t>Dag_Low</t>
+  </si>
+  <si>
+    <t>Dag_Medium</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -165,6 +168,11 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
       <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -211,11 +219,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -551,9 +560,9 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B10"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -561,7 +570,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -569,7 +578,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>3</v>
       </c>
@@ -577,7 +586,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -585,7 +594,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -593,7 +602,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
         <v>9</v>
       </c>
@@ -609,12 +618,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:M12"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="16.53125" customWidth="1"/>
+    <col min="1" max="1" width="16.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -655,7 +664,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -696,7 +705,7 @@
         <v>-1.3359609148359927E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -737,7 +746,7 @@
         <v>-7.2277855207773675E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -778,7 +787,7 @@
         <v>1.6684656836818469E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>29</v>
       </c>
@@ -819,7 +828,7 @@
         <v>-2.0099407435794974E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>30</v>
       </c>
@@ -860,7 +869,7 @@
         <v>-1.3199881490738653E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>31</v>
       </c>
@@ -901,7 +910,7 @@
         <v>-2.3492937485129518E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>32</v>
       </c>
@@ -942,7 +951,7 @@
         <v>-1.2950633218948662E-3</v>
       </c>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>15</v>
       </c>
@@ -983,7 +992,7 @@
         <v>-3.8626841323309791E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>16</v>
       </c>
@@ -1024,7 +1033,7 @@
         <v>5.0088271207424572E-4</v>
       </c>
     </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -1065,7 +1074,7 @@
         <v>-4.2876388871140479E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:13" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>18</v>
       </c>
@@ -1114,12 +1123,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:R17"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="25.265625" customWidth="1"/>
+    <col min="1" max="1" width="25.33203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>10</v>
       </c>
@@ -1175,7 +1184,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>12</v>
       </c>
@@ -1231,7 +1240,7 @@
         <v>-3.4126254766013507E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>13</v>
       </c>
@@ -1287,7 +1296,7 @@
         <v>-5.1539753384105644E-2</v>
       </c>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>14</v>
       </c>
@@ -1343,7 +1352,7 @@
         <v>9.4505907422043236E-4</v>
       </c>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>19</v>
       </c>
@@ -1399,7 +1408,7 @@
         <v>1.8663959943310813E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>20</v>
       </c>
@@ -1455,7 +1464,7 @@
         <v>-9.4429115965450096E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>21</v>
       </c>
@@ -1511,7 +1520,7 @@
         <v>-2.3590724324437824E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>22</v>
       </c>
@@ -1567,7 +1576,7 @@
         <v>6.5198187941972589E-4</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>23</v>
       </c>
@@ -1623,7 +1632,7 @@
         <v>9.0076524435265398E-3</v>
       </c>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>29</v>
       </c>
@@ -1679,7 +1688,7 @@
         <v>4.6190788354832949E-3</v>
       </c>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>30</v>
       </c>
@@ -1735,7 +1744,7 @@
         <v>6.5693578990619669E-3</v>
       </c>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>31</v>
       </c>
@@ -1791,7 +1800,7 @@
         <v>6.7678432814534655E-3</v>
       </c>
     </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>32</v>
       </c>
@@ -1847,7 +1856,7 @@
         <v>1.0544468102314164E-3</v>
       </c>
     </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>15</v>
       </c>
@@ -1903,7 +1912,7 @@
         <v>-8.0760920427191962E-5</v>
       </c>
     </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>16</v>
       </c>
@@ -1959,7 +1968,7 @@
         <v>-4.1003434434182043E-3</v>
       </c>
     </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>17</v>
       </c>
@@ -2015,7 +2024,7 @@
         <v>-9.8739195725258272E-3</v>
       </c>
     </row>
-    <row r="17" spans="1:18" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:18" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -2078,583 +2087,669 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
-  <dimension ref="A1:N13"/>
-  <sheetFormatPr defaultColWidth="8.86328125" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
+  <dimension ref="A1:O14"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="22.86328125" customWidth="1"/>
-    <col min="2" max="2" width="13.265625" customWidth="1"/>
-    <col min="10" max="10" width="20.06640625" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
+    <col min="2" max="2" width="13.33203125" customWidth="1"/>
+    <col min="10" max="10" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A1" t="s">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A1" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E1" t="s">
-        <v>34</v>
-      </c>
-      <c r="F1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H1" t="s">
-        <v>37</v>
-      </c>
-      <c r="I1" t="s">
-        <v>38</v>
-      </c>
-      <c r="J1" t="s">
-        <v>39</v>
-      </c>
-      <c r="K1" t="s">
-        <v>26</v>
-      </c>
-      <c r="L1" t="s">
-        <v>27</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="M1" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="O1" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="2" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="4">
         <v>-0.19475685081635269</v>
       </c>
       <c r="C2">
         <v>1.3409123708389424E-2</v>
       </c>
       <c r="D2">
+        <v>2.1576896824549521E-5</v>
+      </c>
+      <c r="E2">
+        <v>2.9127905724396839E-3</v>
+      </c>
+      <c r="F2">
+        <v>7.590689442179921E-4</v>
+      </c>
+      <c r="G2">
+        <v>1.7422960648879335E-4</v>
+      </c>
+      <c r="H2">
+        <v>7.6344826969746251E-4</v>
+      </c>
+      <c r="I2">
+        <v>9.843075038158493E-5</v>
+      </c>
+      <c r="J2">
+        <v>1.4115207494679497E-4</v>
+      </c>
+      <c r="K2">
+        <v>-2.8238345284652662E-3</v>
+      </c>
+      <c r="L2">
         <v>-9.2143051036281342E-4</v>
-      </c>
-      <c r="E2">
-        <v>2.1576896824549521E-5</v>
-      </c>
-      <c r="F2">
-        <v>2.9127905724396839E-3</v>
-      </c>
-      <c r="G2">
-        <v>7.590689442179921E-4</v>
-      </c>
-      <c r="H2">
-        <v>1.7422960648879335E-4</v>
-      </c>
-      <c r="I2">
-        <v>7.6344826969746251E-4</v>
-      </c>
-      <c r="J2">
-        <v>9.843075038158493E-5</v>
-      </c>
-      <c r="K2">
-        <v>1.4115207494679497E-4</v>
-      </c>
-      <c r="L2">
-        <v>-2.8238345284652662E-3</v>
       </c>
       <c r="M2">
         <v>-6.5626185107372191E-4</v>
       </c>
       <c r="N2">
+        <v>-9.0485190649986424E-4</v>
+      </c>
+      <c r="O2">
         <v>1.6080806168536667E-3</v>
       </c>
     </row>
-    <row r="3" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A3" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B3" s="4">
+        <v>-5.5563641405503239E-2</v>
+      </c>
+      <c r="C3">
+        <v>2.1576896824549521E-5</v>
+      </c>
+      <c r="D3">
+        <v>9.4364827372930198E-5</v>
+      </c>
+      <c r="E3">
+        <v>-1.7608613444121315E-4</v>
+      </c>
+      <c r="F3">
+        <v>1.3714411702458627E-4</v>
+      </c>
+      <c r="G3">
+        <v>-1.6527567791614628E-6</v>
+      </c>
+      <c r="H3">
+        <v>-9.1313247325957442E-6</v>
+      </c>
+      <c r="I3">
+        <v>-7.7886325005704742E-6</v>
+      </c>
+      <c r="J3">
+        <v>-1.6533215482391738E-4</v>
+      </c>
+      <c r="K3">
+        <v>-1.4305423316045458E-4</v>
+      </c>
+      <c r="L3">
+        <v>-4.069997414187055E-3</v>
+      </c>
+      <c r="M3">
+        <v>4.3427464948995548E-2</v>
+      </c>
+      <c r="N3">
+        <v>-4.4294521495035696E-3</v>
+      </c>
+      <c r="O3">
+        <v>5.1751452567861234E-2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="B4" s="4">
+        <v>-0.60866789995718118</v>
+      </c>
+      <c r="C4">
+        <v>2.9127905724396839E-3</v>
+      </c>
+      <c r="D4">
+        <v>-1.7608613444121315E-4</v>
+      </c>
+      <c r="E4">
+        <v>2.9927155670560233E-2</v>
+      </c>
+      <c r="F4">
+        <v>1.6379728915963614E-2</v>
+      </c>
+      <c r="G4">
+        <v>1.5504687985643029E-2</v>
+      </c>
+      <c r="H4">
+        <v>1.6277254518985727E-2</v>
+      </c>
+      <c r="I4">
+        <v>5.0716817343063368E-5</v>
+      </c>
+      <c r="J4">
+        <v>1.5455314641815753E-3</v>
+      </c>
+      <c r="K4">
+        <v>4.0685488155021475E-3</v>
+      </c>
+      <c r="L4">
+        <v>6.810199211806367E-3</v>
+      </c>
+      <c r="M4">
+        <v>-8.456836762273226E-2</v>
+      </c>
+      <c r="N4">
+        <v>7.2602172131255079E-3</v>
+      </c>
+      <c r="O4">
+        <v>-9.0028535514479049E-2</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B5" s="4">
+        <v>-0.70324366588634069</v>
+      </c>
+      <c r="C5">
+        <v>7.590689442179921E-4</v>
+      </c>
+      <c r="D5">
+        <v>1.3714411702458627E-4</v>
+      </c>
+      <c r="E5">
+        <v>1.6379728915963614E-2</v>
+      </c>
+      <c r="F5">
+        <v>4.4022227139688515E-2</v>
+      </c>
+      <c r="G5">
+        <v>1.5621390335502134E-2</v>
+      </c>
+      <c r="H5">
+        <v>1.5972370954907458E-2</v>
+      </c>
+      <c r="I5">
+        <v>5.5134637278203493E-5</v>
+      </c>
+      <c r="J5">
+        <v>-6.7291293666023062E-4</v>
+      </c>
+      <c r="K5">
+        <v>7.3454735056977406E-3</v>
+      </c>
+      <c r="L5">
+        <v>-5.8090593335331821E-3</v>
+      </c>
+      <c r="M5">
+        <v>4.2720539798672852E-2</v>
+      </c>
+      <c r="N5">
+        <v>-7.0623214131569807E-3</v>
+      </c>
+      <c r="O5">
+        <v>7.3753253703915014E-2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="B6" s="4">
+        <v>0.42000823658457415</v>
+      </c>
+      <c r="C6">
+        <v>1.7422960648879335E-4</v>
+      </c>
+      <c r="D6">
+        <v>-1.6527567791614628E-6</v>
+      </c>
+      <c r="E6">
+        <v>1.5504687985643029E-2</v>
+      </c>
+      <c r="F6">
+        <v>1.5621390335502134E-2</v>
+      </c>
+      <c r="G6">
+        <v>2.9378407483991294E-2</v>
+      </c>
+      <c r="H6">
+        <v>1.600243822879166E-2</v>
+      </c>
+      <c r="I6">
+        <v>-3.1583697777708814E-4</v>
+      </c>
+      <c r="J6">
+        <v>-3.0196271770003126E-4</v>
+      </c>
+      <c r="K6">
+        <v>2.5851565590439807E-3</v>
+      </c>
+      <c r="L6">
+        <v>-1.646121953855495E-4</v>
+      </c>
+      <c r="M6">
+        <v>-6.2211762017819958E-3</v>
+      </c>
+      <c r="N6">
+        <v>5.2558639108341455E-4</v>
+      </c>
+      <c r="O6">
+        <v>-2.3582040298859908E-2</v>
+      </c>
+    </row>
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="B7" s="4">
+        <v>-0.12703292623853815</v>
+      </c>
+      <c r="C7">
+        <v>7.6344826969746251E-4</v>
+      </c>
+      <c r="D7">
+        <v>-9.1313247325957442E-6</v>
+      </c>
+      <c r="E7">
+        <v>1.6277254518985727E-2</v>
+      </c>
+      <c r="F7">
+        <v>1.5972370954907458E-2</v>
+      </c>
+      <c r="G7">
+        <v>1.600243822879166E-2</v>
+      </c>
+      <c r="H7">
+        <v>2.8194910082764035E-2</v>
+      </c>
+      <c r="I7">
+        <v>-2.9840957813235158E-4</v>
+      </c>
+      <c r="J7">
+        <v>-4.8818753259096542E-4</v>
+      </c>
+      <c r="K7">
+        <v>3.5584930954063519E-3</v>
+      </c>
+      <c r="L7">
+        <v>-2.3329930256899001E-4</v>
+      </c>
+      <c r="M7">
+        <v>-2.8467612703106659E-3</v>
+      </c>
+      <c r="N7">
+        <v>-3.8159618061404423E-5</v>
+      </c>
+      <c r="O7">
+        <v>-5.8122855107039101E-3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="B8" s="4">
+        <v>-6.0248291948669666E-2</v>
+      </c>
+      <c r="C8">
+        <v>9.843075038158493E-5</v>
+      </c>
+      <c r="D8">
+        <v>-7.7886325005704742E-6</v>
+      </c>
+      <c r="E8">
+        <v>5.0716817343063368E-5</v>
+      </c>
+      <c r="F8">
+        <v>5.5134637278203493E-5</v>
+      </c>
+      <c r="G8">
+        <v>-3.1583697777708814E-4</v>
+      </c>
+      <c r="H8">
+        <v>-2.9840957813235158E-4</v>
+      </c>
+      <c r="I8">
+        <v>3.2266894705745256E-4</v>
+      </c>
+      <c r="J8">
+        <v>-1.5890851266514414E-3</v>
+      </c>
+      <c r="K8">
+        <v>-1.958201772702521E-3</v>
+      </c>
+      <c r="L8">
+        <v>2.8625146749584884E-4</v>
+      </c>
+      <c r="M8">
+        <v>-7.47212173378577E-3</v>
+      </c>
+      <c r="N8">
+        <v>3.0554670858922025E-4</v>
+      </c>
+      <c r="O8">
+        <v>-7.575077380311197E-3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="B9" s="4">
+        <v>0.12532596776269456</v>
+      </c>
+      <c r="C9">
+        <v>1.4115207494679497E-4</v>
+      </c>
+      <c r="D9">
+        <v>-1.6533215482391738E-4</v>
+      </c>
+      <c r="E9">
+        <v>1.5455314641815753E-3</v>
+      </c>
+      <c r="F9">
+        <v>-6.7291293666023062E-4</v>
+      </c>
+      <c r="G9">
+        <v>-3.0196271770003126E-4</v>
+      </c>
+      <c r="H9">
+        <v>-4.8818753259096542E-4</v>
+      </c>
+      <c r="I9">
+        <v>-1.5890851266514414E-3</v>
+      </c>
+      <c r="J9">
+        <v>5.5472330377570732E-2</v>
+      </c>
+      <c r="K9">
+        <v>1.1412873152831213E-2</v>
+      </c>
+      <c r="L9">
+        <v>7.1361350383652711E-3</v>
+      </c>
+      <c r="M9">
+        <v>-5.6170545883362594E-2</v>
+      </c>
+      <c r="N9">
+        <v>7.7771235852395811E-3</v>
+      </c>
+      <c r="O9">
+        <v>-6.9655217486060406E-2</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="B10" s="4">
+        <v>1.2255113266353119</v>
+      </c>
+      <c r="C10">
+        <v>-2.8238345284652662E-3</v>
+      </c>
+      <c r="D10">
+        <v>-1.4305423316045458E-4</v>
+      </c>
+      <c r="E10">
+        <v>4.0685488155021475E-3</v>
+      </c>
+      <c r="F10">
+        <v>7.3454735056977406E-3</v>
+      </c>
+      <c r="G10">
+        <v>2.5851565590439807E-3</v>
+      </c>
+      <c r="H10">
+        <v>3.5584930954063519E-3</v>
+      </c>
+      <c r="I10">
+        <v>-1.958201772702521E-3</v>
+      </c>
+      <c r="J10">
+        <v>1.1412873152831213E-2</v>
+      </c>
+      <c r="K10">
+        <v>0.20402924290055638</v>
+      </c>
+      <c r="L10">
+        <v>6.0308263338469947E-3</v>
+      </c>
+      <c r="M10">
+        <v>-3.6383421002764219E-2</v>
+      </c>
+      <c r="N10">
+        <v>7.2281855639998293E-3</v>
+      </c>
+      <c r="O10">
+        <v>-6.8713031914267558E-2</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B3">
+      <c r="B11" s="4">
         <v>3.0179729767868051</v>
       </c>
-      <c r="C3">
+      <c r="C11">
         <v>-9.2143051036281342E-4</v>
       </c>
-      <c r="D3">
+      <c r="D11">
+        <v>-4.069997414187055E-3</v>
+      </c>
+      <c r="E11">
+        <v>6.810199211806367E-3</v>
+      </c>
+      <c r="F11">
+        <v>-5.8090593335331821E-3</v>
+      </c>
+      <c r="G11">
+        <v>-1.646121953855495E-4</v>
+      </c>
+      <c r="H11">
+        <v>-2.3329930256899001E-4</v>
+      </c>
+      <c r="I11">
+        <v>2.8625146749584884E-4</v>
+      </c>
+      <c r="J11">
+        <v>7.1361350383652711E-3</v>
+      </c>
+      <c r="K11">
+        <v>6.0308263338469947E-3</v>
+      </c>
+      <c r="L11">
         <v>0.17666099300091753</v>
       </c>
-      <c r="E3">
-        <v>-4.069997414187055E-3</v>
-      </c>
-      <c r="F3">
-        <v>6.810199211806367E-3</v>
-      </c>
-      <c r="G3">
-        <v>-5.8090593335331821E-3</v>
-      </c>
-      <c r="H3">
-        <v>-1.646121953855495E-4</v>
-      </c>
-      <c r="I3">
-        <v>-2.3329930256899001E-4</v>
-      </c>
-      <c r="J3">
-        <v>2.8625146749584884E-4</v>
-      </c>
-      <c r="K3">
-        <v>7.1361350383652711E-3</v>
-      </c>
-      <c r="L3">
-        <v>6.0308263338469947E-3</v>
-      </c>
-      <c r="M3">
+      <c r="M11">
         <v>-1.8943742662098764</v>
       </c>
-      <c r="N3">
+      <c r="N11">
+        <v>0.19122788087141718</v>
+      </c>
+      <c r="O11">
         <v>-2.2350063256210682</v>
       </c>
     </row>
-    <row r="4" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B4">
-        <v>-5.5563641405503239E-2</v>
-      </c>
-      <c r="C4">
-        <v>2.1576896824549521E-5</v>
-      </c>
-      <c r="D4">
-        <v>-4.069997414187055E-3</v>
-      </c>
-      <c r="E4">
-        <v>9.4364827372930198E-5</v>
-      </c>
-      <c r="F4">
-        <v>-1.7608613444121315E-4</v>
-      </c>
-      <c r="G4">
-        <v>1.3714411702458627E-4</v>
-      </c>
-      <c r="H4">
-        <v>-1.6527567791614628E-6</v>
-      </c>
-      <c r="I4">
-        <v>-9.1313247325957442E-6</v>
-      </c>
-      <c r="J4">
-        <v>-7.7886325005704742E-6</v>
-      </c>
-      <c r="K4">
-        <v>-1.6533215482391738E-4</v>
-      </c>
-      <c r="L4">
-        <v>-1.4305423316045458E-4</v>
-      </c>
-      <c r="M4">
-        <v>4.3427464948995548E-2</v>
-      </c>
-      <c r="N4">
-        <v>5.1751452567861234E-2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B5">
-        <v>-0.60866789995718118</v>
-      </c>
-      <c r="C5">
-        <v>2.9127905724396839E-3</v>
-      </c>
-      <c r="D5">
-        <v>6.810199211806367E-3</v>
-      </c>
-      <c r="E5">
-        <v>-1.7608613444121315E-4</v>
-      </c>
-      <c r="F5">
-        <v>2.9927155670560233E-2</v>
-      </c>
-      <c r="G5">
-        <v>1.6379728915963614E-2</v>
-      </c>
-      <c r="H5">
-        <v>1.5504687985643029E-2</v>
-      </c>
-      <c r="I5">
-        <v>1.6277254518985727E-2</v>
-      </c>
-      <c r="J5">
-        <v>5.0716817343063368E-5</v>
-      </c>
-      <c r="K5">
-        <v>1.5455314641815753E-3</v>
-      </c>
-      <c r="L5">
-        <v>4.0685488155021475E-3</v>
-      </c>
-      <c r="M5">
-        <v>-8.456836762273226E-2</v>
-      </c>
-      <c r="N5">
-        <v>-9.0028535514479049E-2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6">
-        <v>-0.70324366588634069</v>
-      </c>
-      <c r="C6">
-        <v>7.590689442179921E-4</v>
-      </c>
-      <c r="D6">
-        <v>-5.8090593335331821E-3</v>
-      </c>
-      <c r="E6">
-        <v>1.3714411702458627E-4</v>
-      </c>
-      <c r="F6">
-        <v>1.6379728915963614E-2</v>
-      </c>
-      <c r="G6">
-        <v>4.4022227139688515E-2</v>
-      </c>
-      <c r="H6">
-        <v>1.5621390335502134E-2</v>
-      </c>
-      <c r="I6">
-        <v>1.5972370954907458E-2</v>
-      </c>
-      <c r="J6">
-        <v>5.5134637278203493E-5</v>
-      </c>
-      <c r="K6">
-        <v>-6.7291293666023062E-4</v>
-      </c>
-      <c r="L6">
-        <v>7.3454735056977406E-3</v>
-      </c>
-      <c r="M6">
-        <v>4.2720539798672852E-2</v>
-      </c>
-      <c r="N6">
-        <v>7.3753253703915014E-2</v>
-      </c>
-    </row>
-    <row r="7" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A7" t="s">
-        <v>37</v>
-      </c>
-      <c r="B7">
-        <v>0.42000823658457415</v>
-      </c>
-      <c r="C7">
-        <v>1.7422960648879335E-4</v>
-      </c>
-      <c r="D7">
-        <v>-1.646121953855495E-4</v>
-      </c>
-      <c r="E7">
-        <v>-1.6527567791614628E-6</v>
-      </c>
-      <c r="F7">
-        <v>1.5504687985643029E-2</v>
-      </c>
-      <c r="G7">
-        <v>1.5621390335502134E-2</v>
-      </c>
-      <c r="H7">
-        <v>2.9378407483991294E-2</v>
-      </c>
-      <c r="I7">
-        <v>1.600243822879166E-2</v>
-      </c>
-      <c r="J7">
-        <v>-3.1583697777708814E-4</v>
-      </c>
-      <c r="K7">
-        <v>-3.0196271770003126E-4</v>
-      </c>
-      <c r="L7">
-        <v>2.5851565590439807E-3</v>
-      </c>
-      <c r="M7">
-        <v>-6.2211762017819958E-3</v>
-      </c>
-      <c r="N7">
-        <v>-2.3582040298859908E-2</v>
-      </c>
-    </row>
-    <row r="8" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A8" t="s">
-        <v>38</v>
-      </c>
-      <c r="B8">
-        <v>-0.12703292623853815</v>
-      </c>
-      <c r="C8">
-        <v>7.6344826969746251E-4</v>
-      </c>
-      <c r="D8">
-        <v>-2.3329930256899001E-4</v>
-      </c>
-      <c r="E8">
-        <v>-9.1313247325957442E-6</v>
-      </c>
-      <c r="F8">
-        <v>1.6277254518985727E-2</v>
-      </c>
-      <c r="G8">
-        <v>1.5972370954907458E-2</v>
-      </c>
-      <c r="H8">
-        <v>1.600243822879166E-2</v>
-      </c>
-      <c r="I8">
-        <v>2.8194910082764035E-2</v>
-      </c>
-      <c r="J8">
-        <v>-2.9840957813235158E-4</v>
-      </c>
-      <c r="K8">
-        <v>-4.8818753259096542E-4</v>
-      </c>
-      <c r="L8">
-        <v>3.5584930954063519E-3</v>
-      </c>
-      <c r="M8">
-        <v>-2.8467612703106659E-3</v>
-      </c>
-      <c r="N8">
-        <v>-5.8122855107039101E-3</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
-        <v>39</v>
-      </c>
-      <c r="B9">
-        <v>-6.0248291948669666E-2</v>
-      </c>
-      <c r="C9">
-        <v>9.843075038158493E-5</v>
-      </c>
-      <c r="D9">
-        <v>2.8625146749584884E-4</v>
-      </c>
-      <c r="E9">
-        <v>-7.7886325005704742E-6</v>
-      </c>
-      <c r="F9">
-        <v>5.0716817343063368E-5</v>
-      </c>
-      <c r="G9">
-        <v>5.5134637278203493E-5</v>
-      </c>
-      <c r="H9">
-        <v>-3.1583697777708814E-4</v>
-      </c>
-      <c r="I9">
-        <v>-2.9840957813235158E-4</v>
-      </c>
-      <c r="J9">
-        <v>3.2266894705745256E-4</v>
-      </c>
-      <c r="K9">
-        <v>-1.5890851266514414E-3</v>
-      </c>
-      <c r="L9">
-        <v>-1.958201772702521E-3</v>
-      </c>
-      <c r="M9">
-        <v>-7.47212173378577E-3</v>
-      </c>
-      <c r="N9">
-        <v>-7.575077380311197E-3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A10" t="s">
-        <v>26</v>
-      </c>
-      <c r="B10">
-        <v>0.12532596776269456</v>
-      </c>
-      <c r="C10">
-        <v>1.4115207494679497E-4</v>
-      </c>
-      <c r="D10">
-        <v>7.1361350383652711E-3</v>
-      </c>
-      <c r="E10">
-        <v>-1.6533215482391738E-4</v>
-      </c>
-      <c r="F10">
-        <v>1.5455314641815753E-3</v>
-      </c>
-      <c r="G10">
-        <v>-6.7291293666023062E-4</v>
-      </c>
-      <c r="H10">
-        <v>-3.0196271770003126E-4</v>
-      </c>
-      <c r="I10">
-        <v>-4.8818753259096542E-4</v>
-      </c>
-      <c r="J10">
-        <v>-1.5890851266514414E-3</v>
-      </c>
-      <c r="K10">
-        <v>5.5472330377570732E-2</v>
-      </c>
-      <c r="L10">
-        <v>1.1412873152831213E-2</v>
-      </c>
-      <c r="M10">
-        <v>-5.6170545883362594E-2</v>
-      </c>
-      <c r="N10">
-        <v>-6.9655217486060406E-2</v>
-      </c>
-    </row>
-    <row r="11" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A11" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11">
-        <v>1.2255113266353119</v>
-      </c>
-      <c r="C11">
-        <v>-2.8238345284652662E-3</v>
-      </c>
-      <c r="D11">
-        <v>6.0308263338469947E-3</v>
-      </c>
-      <c r="E11">
-        <v>-1.4305423316045458E-4</v>
-      </c>
-      <c r="F11">
-        <v>4.0685488155021475E-3</v>
-      </c>
-      <c r="G11">
-        <v>7.3454735056977406E-3</v>
-      </c>
-      <c r="H11">
-        <v>2.5851565590439807E-3</v>
-      </c>
-      <c r="I11">
-        <v>3.5584930954063519E-3</v>
-      </c>
-      <c r="J11">
-        <v>-1.958201772702521E-3</v>
-      </c>
-      <c r="K11">
-        <v>1.1412873152831213E-2</v>
-      </c>
-      <c r="L11">
-        <v>0.20402924290055638</v>
-      </c>
-      <c r="M11">
-        <v>-3.6383421002764219E-2</v>
-      </c>
-      <c r="N11">
-        <v>-6.8713031914267558E-2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A12" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B12">
+      <c r="B12" s="4">
         <v>-35.999775981072666</v>
       </c>
       <c r="C12">
         <v>-6.5626185107372191E-4</v>
       </c>
       <c r="D12">
+        <v>4.3427464948995548E-2</v>
+      </c>
+      <c r="E12">
+        <v>-8.456836762273226E-2</v>
+      </c>
+      <c r="F12">
+        <v>4.2720539798672852E-2</v>
+      </c>
+      <c r="G12">
+        <v>-6.2211762017819958E-3</v>
+      </c>
+      <c r="H12">
+        <v>-2.8467612703106659E-3</v>
+      </c>
+      <c r="I12">
+        <v>-7.47212173378577E-3</v>
+      </c>
+      <c r="J12">
+        <v>-5.6170545883362594E-2</v>
+      </c>
+      <c r="K12">
+        <v>-3.6383421002764219E-2</v>
+      </c>
+      <c r="L12">
         <v>-1.8943742662098764</v>
-      </c>
-      <c r="E12">
-        <v>4.3427464948995548E-2</v>
-      </c>
-      <c r="F12">
-        <v>-8.456836762273226E-2</v>
-      </c>
-      <c r="G12">
-        <v>4.2720539798672852E-2</v>
-      </c>
-      <c r="H12">
-        <v>-6.2211762017819958E-3</v>
-      </c>
-      <c r="I12">
-        <v>-2.8467612703106659E-3</v>
-      </c>
-      <c r="J12">
-        <v>-7.47212173378577E-3</v>
-      </c>
-      <c r="K12">
-        <v>-5.6170545883362594E-2</v>
-      </c>
-      <c r="L12">
-        <v>-3.6383421002764219E-2</v>
       </c>
       <c r="M12">
         <v>20.488600015981518</v>
       </c>
       <c r="N12">
+        <v>-2.0408408628839201</v>
+      </c>
+      <c r="O12">
         <v>23.932897346374034</v>
       </c>
     </row>
-    <row r="13" spans="1:14" x14ac:dyDescent="0.45">
-      <c r="A13" t="s">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="B13" s="4">
+        <v>3.463843445576031</v>
+      </c>
+      <c r="C13">
+        <v>-9.0485190649986424E-4</v>
+      </c>
+      <c r="D13">
+        <v>-4.4294521495035696E-3</v>
+      </c>
+      <c r="E13">
+        <v>7.2602172131255079E-3</v>
+      </c>
+      <c r="F13">
+        <v>-7.0623214131569807E-3</v>
+      </c>
+      <c r="G13">
+        <v>5.2558639108341455E-4</v>
+      </c>
+      <c r="H13">
+        <v>-3.8159618061404423E-5</v>
+      </c>
+      <c r="I13">
+        <v>3.0554670858922025E-4</v>
+      </c>
+      <c r="J13">
+        <v>7.7771235852395811E-3</v>
+      </c>
+      <c r="K13">
+        <v>7.2281855639998293E-3</v>
+      </c>
+      <c r="L13">
+        <v>0.19122788087141718</v>
+      </c>
+      <c r="M13">
+        <v>-2.0408408628839201</v>
+      </c>
+      <c r="N13">
+        <v>0.20978342293176833</v>
+      </c>
+      <c r="O13">
+        <v>-2.4733730279631736</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="B13">
+      <c r="B14" s="4">
         <v>-50.492821427610203</v>
       </c>
-      <c r="C13">
+      <c r="C14">
         <v>1.6080806168536667E-3</v>
       </c>
-      <c r="D13">
+      <c r="D14">
+        <v>5.1751452567861234E-2</v>
+      </c>
+      <c r="E14">
+        <v>-9.0028535514479049E-2</v>
+      </c>
+      <c r="F14">
+        <v>7.3753253703915014E-2</v>
+      </c>
+      <c r="G14">
+        <v>-2.3582040298859908E-2</v>
+      </c>
+      <c r="H14">
+        <v>-5.8122855107039101E-3</v>
+      </c>
+      <c r="I14">
+        <v>-7.575077380311197E-3</v>
+      </c>
+      <c r="J14">
+        <v>-6.9655217486060406E-2</v>
+      </c>
+      <c r="K14">
+        <v>-6.8713031914267558E-2</v>
+      </c>
+      <c r="L14">
         <v>-2.2350063256210682</v>
       </c>
-      <c r="E13">
-        <v>5.1751452567861234E-2</v>
-      </c>
-      <c r="F13">
-        <v>-9.0028535514479049E-2</v>
-      </c>
-      <c r="G13">
-        <v>7.3753253703915014E-2</v>
-      </c>
-      <c r="H13">
-        <v>-2.3582040298859908E-2</v>
-      </c>
-      <c r="I13">
-        <v>-5.8122855107039101E-3</v>
-      </c>
-      <c r="J13">
-        <v>-7.575077380311197E-3</v>
-      </c>
-      <c r="K13">
-        <v>-6.9655217486060406E-2</v>
-      </c>
-      <c r="L13">
-        <v>-6.8713031914267558E-2</v>
-      </c>
-      <c r="M13">
+      <c r="M14">
         <v>23.932897346374034</v>
       </c>
-      <c r="N13">
+      <c r="N14">
+        <v>-2.4733730279631736</v>
+      </c>
+      <c r="O14">
         <v>29.51973160464496</v>
       </c>
     </row>

</xml_diff>